<commit_message>
Update France Fnac Samsung OLED (18 models) and Micro RGB (4 models) survey data
</commit_message>
<xml_diff>
--- a/data/price tracker_EU_2026 0811_v1.xlsx
+++ b/data/price tracker_EU_2026 0811_v1.xlsx
@@ -7073,7 +7073,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7151,7 +7151,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>784.41</v>
+        <v>839.99</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -7334,19 +7334,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>QLED</t>
+          <t>OLED</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>TQ50Q7F</t>
+          <t>TQ48S90F</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>459.99</v>
+        <v>809</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -7369,23 +7369,23 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Neo QLED</t>
+          <t>OLED</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>TQ50QN90F</t>
+          <t>TQ48S95H</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>899.99</v>
+        <v>1799</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -7408,11 +7408,11 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LED</t>
+          <t>QLED</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -7420,11 +7420,11 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>TU50M72H</t>
+          <t>TQ50Q7F</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>599.99</v>
+        <v>459.99</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -7447,11 +7447,11 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>UHD 4K</t>
+          <t>Neo QLED</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -7459,11 +7459,11 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>TU50U8005H</t>
+          <t>TQ50QN90F</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>479.99</v>
+        <v>899.99</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -7486,23 +7486,23 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>QLED</t>
+          <t>LED</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>TQ55LS03F</t>
+          <t>TU50M72H</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>100</v>
+        <v>499.99</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -7529,19 +7529,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>QLED</t>
+          <t>UHD 4K</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>TQ55LS03H</t>
+          <t>TU50U8005H</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1399</v>
+        <v>479.99</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -7564,7 +7564,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -7576,11 +7576,11 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>TQ55LS03HW</t>
+          <t>TQ55LS03F</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1499</v>
+        <v>829.99</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -7603,7 +7603,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -7615,11 +7615,11 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>TQ55Q6F</t>
+          <t>TQ55LS03H</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>382.49</v>
+        <v>1399</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -7642,7 +7642,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -7654,11 +7654,11 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>TQ55Q7F5</t>
+          <t>TQ55LS03HW</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>475.79</v>
+        <v>1499</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -7681,11 +7681,11 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Neo QLED</t>
+          <t>QLED</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -7693,11 +7693,11 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>TQ55QN74H</t>
+          <t>TQ55Q6F</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>799.99</v>
+        <v>382.49</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -7720,11 +7720,11 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Neo QLED</t>
+          <t>QLED</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -7732,11 +7732,11 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>TQ55QN82H</t>
+          <t>TQ55Q7F5</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>1199</v>
+        <v>479.99</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -7759,11 +7759,11 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>OLED</t>
+          <t>Neo QLED</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -7771,11 +7771,11 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>TQ55S90F</t>
+          <t>TQ55QN74H</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>888</v>
+        <v>799.99</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -7802,7 +7802,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>OLED</t>
+          <t>Neo QLED</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -7810,11 +7810,11 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>TQ55S95H</t>
+          <t>TQ55QN82H</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2099</v>
+        <v>1199</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -7837,7 +7837,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -7849,11 +7849,11 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>TQ55S99H</t>
+          <t>TQ55S90F</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2499</v>
+        <v>989</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -7880,7 +7880,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>LED</t>
+          <t>OLED</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -7888,11 +7888,11 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>TU55M80H</t>
+          <t>TQ55S92H</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>699.99</v>
+        <v>1899</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -7915,11 +7915,11 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>UHD 4K</t>
+          <t>OLED</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -7927,11 +7927,11 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>TU55U8005H</t>
+          <t>TQ55S95F</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>529.99</v>
+        <v>1499</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -7954,23 +7954,23 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>QLED</t>
+          <t>OLED</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>TQ65LS03FW</t>
+          <t>TQ55S95H</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>100</v>
+        <v>2099</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -7993,23 +7993,23 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>QLED</t>
+          <t>OLED</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>TQ65Q7F</t>
+          <t>TQ55S99H</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>594.29</v>
+        <v>2499</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -8032,23 +8032,23 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Neo QLED</t>
+          <t>LED</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>TQ65QN74F</t>
+          <t>TU55M80H</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>689.99</v>
+        <v>699.99</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -8075,19 +8075,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Neo QLED</t>
+          <t>UHD 4K</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>TQ65QN82H</t>
+          <t>TU55U8005H</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>100</v>
+        <v>529.99</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -8110,11 +8110,11 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Neo QLED</t>
+          <t>LED</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -8122,11 +8122,11 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>TQ65QN85F</t>
+          <t>TMR65R85H</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>799</v>
+        <v>1999</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -8153,7 +8153,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>OLED</t>
+          <t>LED</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -8161,11 +8161,11 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>TQ65S92H</t>
+          <t>TMR65R95H</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>100</v>
+        <v>3799</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -8192,7 +8192,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>OLED</t>
+          <t>QLED</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -8200,11 +8200,11 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>TQ65S95F</t>
+          <t>TQ65LS03FW</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>100</v>
+        <v>1199</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -8227,11 +8227,11 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>OLED</t>
+          <t>QLED</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -8239,11 +8239,11 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>TQ65S99H</t>
+          <t>TQ65Q6F</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3499</v>
+        <v>588.29</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -8266,11 +8266,11 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LED</t>
+          <t>QLED</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -8278,11 +8278,11 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>TU65M80H</t>
+          <t>TQ65Q7F</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>849.99</v>
+        <v>599.99</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -8309,19 +8309,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>QLED</t>
+          <t>Neo QLED</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>27LSM7FA</t>
+          <t>TQ65QN74F</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>999.99</v>
+        <v>689.99</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -8344,23 +8344,23 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>QLED</t>
+          <t>Neo QLED</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>TQ75Q7F</t>
+          <t>TQ65QN82H</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>768.1900000000001</v>
+        <v>1499</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -8391,15 +8391,15 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>TQ75QN74F</t>
+          <t>TQ65QN85F</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>999.99</v>
+        <v>799</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -8426,19 +8426,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Neo QLED</t>
+          <t>OLED</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>TQ75QN85F</t>
+          <t>TQ65S85F</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>891.65</v>
+        <v>1749.81</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -8461,7 +8461,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -8469,15 +8469,15 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>TQ77S95H</t>
+          <t>TQ65S90F</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>100</v>
+        <v>1379</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -8500,23 +8500,23 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>QLED</t>
+          <t>OLED</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>TQ32Q5FA</t>
+          <t>TQ65S92H</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>379.99</v>
+        <v>2599</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -8543,19 +8543,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>QLED</t>
+          <t>OLED</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>TQ85Q7F</t>
+          <t>TQ65S95F</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>979</v>
+        <v>1799</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -8582,19 +8582,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>UHD 4K</t>
+          <t>OLED</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>TU85M80H</t>
+          <t>TQ65S95H</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>1599</v>
+        <v>3669.99</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -8617,33 +8617,735 @@
         </is>
       </c>
       <c r="B40" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>OLED</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>65</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>TQ65S99H</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>3499</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>SAMSUNG</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>LED</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>65</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>TU65M80H</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>849.99</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SAMSUNG</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
         <v>2025</v>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>QLED</t>
         </is>
       </c>
-      <c r="D40" t="n">
+      <c r="D42" t="n">
+        <v>68</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>27LSM7FA</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>999.99</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>SAMSUNG</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>LED</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>75</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>TMR75R85H</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>2499</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>SAMSUNG</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>QLED</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>75</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>TQ75Q7F</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>899.99</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SAMSUNG</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Neo QLED</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>75</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>TQ75QN74F</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>999.99</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>SAMSUNG</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Neo QLED</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>75</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>TQ75QN82H</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>1999</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SAMSUNG</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Neo QLED</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>75</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>TQ75QN85F</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>891.65</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SAMSUNG</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>UHD 4K</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>75</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>TU75U8005H</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>879.99</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>SAMSUNG</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>OLED</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>77</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>TQ77S90F</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>1799</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>SAMSUNG</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>OLED</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>77</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>TQ77S95H</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>4399</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>SAMSUNG</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>OLED</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>77</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>TQ77S99H</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>4499</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>SAMSUNG</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>QLED</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>81</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>TQ32Q5FA</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>379.99</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>SAMSUNG</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>OLED</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>83</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>TQ83S90F</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>2299</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>SAMSUNG</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>LED</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>85</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>TMR85R85H</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>4499</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>SAMSUNG</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>QLED</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>85</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>TQ85Q7F</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>979</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>SAMSUNG</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Neo QLED</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>85</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>TQ85QN74H</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>1799</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>SAMSUNG</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>UHD 4K</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>85</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>TU85M80H</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>1599</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>SAMSUNG</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>QLED</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
         <v>98</v>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E58" t="inlineStr">
         <is>
           <t>TQ98Q7FA</t>
         </is>
       </c>
-      <c r="F40" t="n">
+      <c r="F58" t="n">
         <v>1868.42</v>
       </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="I40" t="n">
-        <v>0</v>
-      </c>
-      <c r="J40" t="inlineStr">
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" t="inlineStr">
         <is>
           <t>None</t>
         </is>

</xml_diff>